<commit_message>
✨ feat(BRB): Add BRB Model
</commit_message>
<xml_diff>
--- a/OutData/push/model_fit_1.50e+03/ModelManager.xlsx
+++ b/OutData/push/model_fit_1.50e+03/ModelManager.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F124"/>
+  <dimension ref="A1:F123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -689,11 +689,11 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>node</t>
+          <t>element</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr"/>
@@ -705,11 +705,11 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>node</t>
+          <t>beamIntegration</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr"/>
@@ -721,11 +721,11 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>node</t>
+          <t>element</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr"/>
@@ -741,7 +741,7 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>43</v>
+        <v>54</v>
       </c>
       <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr"/>
@@ -753,11 +753,11 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>node</t>
+          <t>element</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>40</v>
+        <v>3</v>
       </c>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr"/>
@@ -769,11 +769,11 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>node</t>
+          <t>uniaxialMaterial</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>37</v>
+        <v>11</v>
       </c>
       <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr"/>
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>23</v>
+        <v>48</v>
       </c>
       <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr"/>
@@ -801,11 +801,11 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>node</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>20</v>
+        <v>5</v>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr"/>
@@ -817,11 +817,11 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>node</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr"/>
@@ -833,11 +833,11 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>node</t>
+          <t>element</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr"/>
@@ -849,11 +849,11 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>node</t>
+          <t>element</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>42</v>
+        <v>7</v>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr"/>
@@ -869,7 +869,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr"/>
@@ -885,7 +885,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr"/>
@@ -901,7 +901,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>16</v>
+        <v>4</v>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr"/>
@@ -917,9 +917,13 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>2</v>
-      </c>
-      <c r="D26" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>disp_ctrl</t>
+        </is>
+      </c>
       <c r="E26" t="inlineStr"/>
       <c r="F26" t="inlineStr"/>
     </row>
@@ -929,11 +933,11 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>uniaxialMaterial</t>
+          <t>element</t>
         </is>
       </c>
       <c r="C27" t="n">
-        <v>12</v>
+        <v>33</v>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr"/>
@@ -945,11 +949,11 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>node</t>
         </is>
       </c>
       <c r="C28" t="n">
-        <v>17</v>
+        <v>47</v>
       </c>
       <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr"/>
@@ -965,7 +969,7 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr"/>
@@ -977,17 +981,13 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>node</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>28</v>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>pier_1_ED_2</t>
-        </is>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr"/>
       <c r="F30" t="inlineStr"/>
     </row>
@@ -1001,7 +1001,7 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr"/>
@@ -1013,11 +1013,11 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>node</t>
+          <t>element</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr"/>
@@ -1029,11 +1029,11 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>beamIntegration</t>
+          <t>node</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>2</v>
+        <v>29</v>
       </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr"/>
@@ -1045,11 +1045,11 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>node</t>
+          <t>beamIntegration</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>47</v>
+        <v>1</v>
       </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr"/>
@@ -1061,11 +1061,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>node</t>
+          <t>element</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr"/>
@@ -1081,13 +1081,9 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>27</v>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>pier_1_ED_1</t>
-        </is>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr"/>
       <c r="F36" t="inlineStr"/>
     </row>
@@ -1097,11 +1093,11 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>node</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>50</v>
+        <v>11</v>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr"/>
@@ -1113,11 +1109,11 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>node</t>
+          <t>element</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr"/>
@@ -1133,7 +1129,7 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>55</v>
+        <v>9</v>
       </c>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr"/>
@@ -1149,7 +1145,7 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>31</v>
+        <v>6</v>
       </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr"/>
@@ -1161,19 +1157,23 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>uniaxialMaterial</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>30</v>
+        <v>9</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>pier_2_ED_2</t>
+          <t>PT</t>
         </is>
       </c>
       <c r="E41" t="inlineStr"/>
-      <c r="F41" t="inlineStr"/>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>{'fy': 1860000.0, 'Es': 195000000.0, 'force': 744000.0, 'yield': 0.009538461538461539}</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1181,11 +1181,11 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>node</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>33</v>
+        <v>52</v>
       </c>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr"/>
@@ -1201,7 +1201,7 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>11</v>
+        <v>40</v>
       </c>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr"/>
@@ -1217,7 +1217,7 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D44" t="inlineStr"/>
       <c r="E44" t="inlineStr"/>
@@ -1233,7 +1233,7 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>40</v>
+        <v>22</v>
       </c>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr"/>
@@ -1245,11 +1245,11 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>node</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr"/>
@@ -1261,11 +1261,11 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>node</t>
+          <t>element</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>52</v>
+        <v>24</v>
       </c>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr"/>
@@ -1281,7 +1281,7 @@
         </is>
       </c>
       <c r="C48" t="n">
-        <v>49</v>
+        <v>16</v>
       </c>
       <c r="D48" t="inlineStr"/>
       <c r="E48" t="inlineStr"/>
@@ -1293,11 +1293,11 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>node</t>
+          <t>element</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>35</v>
+        <v>12</v>
       </c>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr"/>
@@ -1309,11 +1309,11 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>node</t>
+          <t>element</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>32</v>
+        <v>9</v>
       </c>
       <c r="D50" t="inlineStr"/>
       <c r="E50" t="inlineStr"/>
@@ -1329,7 +1329,7 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>15</v>
+        <v>50</v>
       </c>
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr"/>
@@ -1345,7 +1345,7 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>33</v>
+        <v>21</v>
       </c>
       <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr"/>
@@ -1357,11 +1357,11 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>node</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>38</v>
+        <v>3</v>
       </c>
       <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr"/>
@@ -1377,9 +1377,13 @@
         </is>
       </c>
       <c r="C54" t="n">
-        <v>2</v>
-      </c>
-      <c r="D54" t="inlineStr"/>
+        <v>30</v>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>pier_2_ED_2</t>
+        </is>
+      </c>
       <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr"/>
     </row>
@@ -1389,15 +1393,15 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>node</t>
+          <t>element</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>1</v>
+        <v>27</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>disp_ctrl</t>
+          <t>pier_1_ED_1</t>
         </is>
       </c>
       <c r="E55" t="inlineStr"/>
@@ -1409,23 +1413,15 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>uniaxialMaterial</t>
+          <t>node</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>9</v>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>PT</t>
-        </is>
-      </c>
+        <v>44</v>
+      </c>
+      <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr"/>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>{'fy': 1860000.0, 'Es': 195000000.0, 'force': 744000.0, 'yield': 0.009538461538461539}</t>
-        </is>
-      </c>
+      <c r="F56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -1433,11 +1429,11 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>node</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr"/>
@@ -1449,13 +1445,17 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>node</t>
+          <t>element</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>5</v>
-      </c>
-      <c r="D58" t="inlineStr"/>
+        <v>37</v>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>pier_1_surf</t>
+        </is>
+      </c>
       <c r="E58" t="inlineStr"/>
       <c r="F58" t="inlineStr"/>
     </row>
@@ -1465,13 +1465,17 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>beamIntegration</t>
+          <t>element</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>1</v>
-      </c>
-      <c r="D59" t="inlineStr"/>
+        <v>32</v>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>PT_2</t>
+        </is>
+      </c>
       <c r="E59" t="inlineStr"/>
       <c r="F59" t="inlineStr"/>
     </row>
@@ -1485,7 +1489,7 @@
         </is>
       </c>
       <c r="C60" t="n">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="D60" t="inlineStr"/>
       <c r="E60" t="inlineStr"/>
@@ -1501,7 +1505,7 @@
         </is>
       </c>
       <c r="C61" t="n">
-        <v>44</v>
+        <v>14</v>
       </c>
       <c r="D61" t="inlineStr"/>
       <c r="E61" t="inlineStr"/>
@@ -1517,7 +1521,7 @@
         </is>
       </c>
       <c r="C62" t="n">
-        <v>46</v>
+        <v>2</v>
       </c>
       <c r="D62" t="inlineStr"/>
       <c r="E62" t="inlineStr"/>
@@ -1529,11 +1533,11 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>node</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>39</v>
+        <v>48</v>
       </c>
       <c r="D63" t="inlineStr"/>
       <c r="E63" t="inlineStr"/>
@@ -1549,7 +1553,7 @@
         </is>
       </c>
       <c r="C64" t="n">
-        <v>24</v>
+        <v>45</v>
       </c>
       <c r="D64" t="inlineStr"/>
       <c r="E64" t="inlineStr"/>
@@ -1561,11 +1565,11 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>node</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>22</v>
+        <v>28</v>
       </c>
       <c r="D65" t="inlineStr"/>
       <c r="E65" t="inlineStr"/>
@@ -1577,11 +1581,11 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>node</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="D66" t="inlineStr"/>
       <c r="E66" t="inlineStr"/>
@@ -1593,11 +1597,11 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>uniaxialMaterial</t>
+          <t>node</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D67" t="inlineStr"/>
       <c r="E67" t="inlineStr"/>
@@ -1613,7 +1617,7 @@
         </is>
       </c>
       <c r="C68" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="D68" t="inlineStr"/>
       <c r="E68" t="inlineStr"/>
@@ -1629,7 +1633,7 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>6</v>
+        <v>49</v>
       </c>
       <c r="D69" t="inlineStr"/>
       <c r="E69" t="inlineStr"/>
@@ -1641,11 +1645,11 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>node</t>
+          <t>element</t>
         </is>
       </c>
       <c r="C70" t="n">
-        <v>4</v>
+        <v>42</v>
       </c>
       <c r="D70" t="inlineStr"/>
       <c r="E70" t="inlineStr"/>
@@ -1661,7 +1665,7 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="D71" t="inlineStr"/>
       <c r="E71" t="inlineStr"/>
@@ -1673,11 +1677,11 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>node</t>
         </is>
       </c>
       <c r="C72" t="n">
-        <v>45</v>
+        <v>10</v>
       </c>
       <c r="D72" t="inlineStr"/>
       <c r="E72" t="inlineStr"/>
@@ -1689,11 +1693,11 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>uniaxialMaterial</t>
         </is>
       </c>
       <c r="C73" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D73" t="inlineStr"/>
       <c r="E73" t="inlineStr"/>
@@ -1709,7 +1713,7 @@
         </is>
       </c>
       <c r="C74" t="n">
-        <v>49</v>
+        <v>19</v>
       </c>
       <c r="D74" t="inlineStr"/>
       <c r="E74" t="inlineStr"/>
@@ -1721,17 +1725,13 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>node</t>
         </is>
       </c>
       <c r="C75" t="n">
-        <v>46</v>
-      </c>
-      <c r="D75" t="inlineStr">
-        <is>
-          <t>pier_2_surf</t>
-        </is>
-      </c>
+        <v>51</v>
+      </c>
+      <c r="D75" t="inlineStr"/>
       <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr"/>
     </row>
@@ -1741,17 +1741,13 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>node</t>
         </is>
       </c>
       <c r="C76" t="n">
-        <v>32</v>
-      </c>
-      <c r="D76" t="inlineStr">
-        <is>
-          <t>PT_2</t>
-        </is>
-      </c>
+        <v>36</v>
+      </c>
+      <c r="D76" t="inlineStr"/>
       <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr"/>
     </row>
@@ -1761,17 +1757,13 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>node</t>
         </is>
       </c>
       <c r="C77" t="n">
-        <v>29</v>
-      </c>
-      <c r="D77" t="inlineStr">
-        <is>
-          <t>pier_2_ED_1</t>
-        </is>
-      </c>
+        <v>33</v>
+      </c>
+      <c r="D77" t="inlineStr"/>
       <c r="E77" t="inlineStr"/>
       <c r="F77" t="inlineStr"/>
     </row>
@@ -1785,7 +1777,7 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>51</v>
+        <v>31</v>
       </c>
       <c r="D78" t="inlineStr"/>
       <c r="E78" t="inlineStr"/>
@@ -1801,7 +1793,7 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>48</v>
+        <v>13</v>
       </c>
       <c r="D79" t="inlineStr"/>
       <c r="E79" t="inlineStr"/>
@@ -1813,11 +1805,11 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>node</t>
+          <t>element</t>
         </is>
       </c>
       <c r="C80" t="n">
-        <v>34</v>
+        <v>6</v>
       </c>
       <c r="D80" t="inlineStr"/>
       <c r="E80" t="inlineStr"/>
@@ -1829,11 +1821,11 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>node</t>
+          <t>element</t>
         </is>
       </c>
       <c r="C81" t="n">
-        <v>29</v>
+        <v>1</v>
       </c>
       <c r="D81" t="inlineStr"/>
       <c r="E81" t="inlineStr"/>
@@ -1845,11 +1837,11 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>node</t>
+          <t>element</t>
         </is>
       </c>
       <c r="C82" t="n">
-        <v>7</v>
+        <v>47</v>
       </c>
       <c r="D82" t="inlineStr"/>
       <c r="E82" t="inlineStr"/>
@@ -1865,7 +1857,7 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>12</v>
+        <v>44</v>
       </c>
       <c r="D83" t="inlineStr"/>
       <c r="E83" t="inlineStr"/>
@@ -1877,11 +1869,11 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>node</t>
         </is>
       </c>
       <c r="C84" t="n">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="D84" t="inlineStr"/>
       <c r="E84" t="inlineStr"/>
@@ -1893,11 +1885,11 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>node</t>
         </is>
       </c>
       <c r="C85" t="n">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="D85" t="inlineStr"/>
       <c r="E85" t="inlineStr"/>
@@ -1909,13 +1901,17 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>node</t>
+          <t>element</t>
         </is>
       </c>
       <c r="C86" t="n">
-        <v>38</v>
-      </c>
-      <c r="D86" t="inlineStr"/>
+        <v>29</v>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>pier_2_ED_1</t>
+        </is>
+      </c>
       <c r="E86" t="inlineStr"/>
       <c r="F86" t="inlineStr"/>
     </row>
@@ -1929,7 +1925,7 @@
         </is>
       </c>
       <c r="C87" t="n">
-        <v>21</v>
+        <v>38</v>
       </c>
       <c r="D87" t="inlineStr"/>
       <c r="E87" t="inlineStr"/>
@@ -1945,7 +1941,7 @@
         </is>
       </c>
       <c r="C88" t="n">
-        <v>18</v>
+        <v>41</v>
       </c>
       <c r="D88" t="inlineStr"/>
       <c r="E88" t="inlineStr"/>
@@ -1961,9 +1957,13 @@
         </is>
       </c>
       <c r="C89" t="n">
-        <v>14</v>
-      </c>
-      <c r="D89" t="inlineStr"/>
+        <v>31</v>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>PT_1</t>
+        </is>
+      </c>
       <c r="E89" t="inlineStr"/>
       <c r="F89" t="inlineStr"/>
     </row>
@@ -1977,7 +1977,7 @@
         </is>
       </c>
       <c r="C90" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="D90" t="inlineStr"/>
       <c r="E90" t="inlineStr"/>
@@ -1989,13 +1989,17 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>node</t>
+          <t>element</t>
         </is>
       </c>
       <c r="C91" t="n">
-        <v>54</v>
-      </c>
-      <c r="D91" t="inlineStr"/>
+        <v>28</v>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>pier_1_ED_2</t>
+        </is>
+      </c>
       <c r="E91" t="inlineStr"/>
       <c r="F91" t="inlineStr"/>
     </row>
@@ -2005,17 +2009,13 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>node</t>
         </is>
       </c>
       <c r="C92" t="n">
-        <v>37</v>
-      </c>
-      <c r="D92" t="inlineStr">
-        <is>
-          <t>pier_1_surf</t>
-        </is>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="D92" t="inlineStr"/>
       <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr"/>
     </row>
@@ -2029,7 +2029,7 @@
         </is>
       </c>
       <c r="C93" t="n">
-        <v>34</v>
+        <v>16</v>
       </c>
       <c r="D93" t="inlineStr"/>
       <c r="E93" t="inlineStr"/>
@@ -2041,11 +2041,11 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>node</t>
+          <t>element</t>
         </is>
       </c>
       <c r="C94" t="n">
-        <v>39</v>
+        <v>11</v>
       </c>
       <c r="D94" t="inlineStr"/>
       <c r="E94" t="inlineStr"/>
@@ -2061,7 +2061,7 @@
         </is>
       </c>
       <c r="C95" t="n">
-        <v>36</v>
+        <v>43</v>
       </c>
       <c r="D95" t="inlineStr"/>
       <c r="E95" t="inlineStr"/>
@@ -2073,11 +2073,11 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>node</t>
+          <t>element</t>
         </is>
       </c>
       <c r="C96" t="n">
-        <v>12</v>
+        <v>49</v>
       </c>
       <c r="D96" t="inlineStr"/>
       <c r="E96" t="inlineStr"/>
@@ -2089,23 +2089,15 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>uniaxialMaterial</t>
+          <t>node</t>
         </is>
       </c>
       <c r="C97" t="n">
-        <v>8</v>
-      </c>
-      <c r="D97" t="inlineStr">
-        <is>
-          <t>ED</t>
-        </is>
-      </c>
+        <v>25</v>
+      </c>
+      <c r="D97" t="inlineStr"/>
       <c r="E97" t="inlineStr"/>
-      <c r="F97" t="inlineStr">
-        <is>
-          <t>{'fy': 437300.0, 'Es': 201000000.0, 'area': 0.00011309733552923255, 'yield': 0.0021756218905472635}</t>
-        </is>
-      </c>
+      <c r="F97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -2113,11 +2105,11 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>node</t>
         </is>
       </c>
       <c r="C98" t="n">
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="D98" t="inlineStr"/>
       <c r="E98" t="inlineStr"/>
@@ -2129,11 +2121,11 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>uniaxialMaterial</t>
+          <t>element</t>
         </is>
       </c>
       <c r="C99" t="n">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="D99" t="inlineStr"/>
       <c r="E99" t="inlineStr"/>
@@ -2145,11 +2137,11 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>node</t>
         </is>
       </c>
       <c r="C100" t="n">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="D100" t="inlineStr"/>
       <c r="E100" t="inlineStr"/>
@@ -2165,7 +2157,7 @@
         </is>
       </c>
       <c r="C101" t="n">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="D101" t="inlineStr"/>
       <c r="E101" t="inlineStr"/>
@@ -2181,7 +2173,7 @@
         </is>
       </c>
       <c r="C102" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D102" t="inlineStr"/>
       <c r="E102" t="inlineStr"/>
@@ -2193,11 +2185,11 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>node</t>
+          <t>element</t>
         </is>
       </c>
       <c r="C103" t="n">
-        <v>23</v>
+        <v>41</v>
       </c>
       <c r="D103" t="inlineStr"/>
       <c r="E103" t="inlineStr"/>
@@ -2209,11 +2201,11 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>node</t>
         </is>
       </c>
       <c r="C104" t="n">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c r="D104" t="inlineStr"/>
       <c r="E104" t="inlineStr"/>
@@ -2229,7 +2221,7 @@
         </is>
       </c>
       <c r="C105" t="n">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="D105" t="inlineStr"/>
       <c r="E105" t="inlineStr"/>
@@ -2245,7 +2237,7 @@
         </is>
       </c>
       <c r="C106" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D106" t="inlineStr"/>
       <c r="E106" t="inlineStr"/>
@@ -2261,7 +2253,7 @@
         </is>
       </c>
       <c r="C107" t="n">
-        <v>3</v>
+        <v>50</v>
       </c>
       <c r="D107" t="inlineStr"/>
       <c r="E107" t="inlineStr"/>
@@ -2277,7 +2269,7 @@
         </is>
       </c>
       <c r="C108" t="n">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="D108" t="inlineStr"/>
       <c r="E108" t="inlineStr"/>
@@ -2289,11 +2281,11 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>node</t>
+          <t>element</t>
         </is>
       </c>
       <c r="C109" t="n">
-        <v>22</v>
+        <v>35</v>
       </c>
       <c r="D109" t="inlineStr"/>
       <c r="E109" t="inlineStr"/>
@@ -2305,11 +2297,11 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>uniaxialMaterial</t>
+          <t>element</t>
         </is>
       </c>
       <c r="C110" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="D110" t="inlineStr"/>
       <c r="E110" t="inlineStr"/>
@@ -2321,15 +2313,23 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>uniaxialMaterial</t>
         </is>
       </c>
       <c r="C111" t="n">
-        <v>48</v>
-      </c>
-      <c r="D111" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>ED</t>
+        </is>
+      </c>
       <c r="E111" t="inlineStr"/>
-      <c r="F111" t="inlineStr"/>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>{'fy': 437300.0, 'Es': 201000000.0, 'area': 0.00011309733552923255, 'yield': 0.0021756218905472635}</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -2337,17 +2337,13 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>uniaxialMaterial</t>
         </is>
       </c>
       <c r="C112" t="n">
-        <v>31</v>
-      </c>
-      <c r="D112" t="inlineStr">
-        <is>
-          <t>PT_1</t>
-        </is>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="D112" t="inlineStr"/>
       <c r="E112" t="inlineStr"/>
       <c r="F112" t="inlineStr"/>
     </row>
@@ -2361,7 +2357,7 @@
         </is>
       </c>
       <c r="C113" t="n">
-        <v>28</v>
+        <v>53</v>
       </c>
       <c r="D113" t="inlineStr"/>
       <c r="E113" t="inlineStr"/>
@@ -2373,13 +2369,17 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>node</t>
+          <t>element</t>
         </is>
       </c>
       <c r="C114" t="n">
-        <v>9</v>
-      </c>
-      <c r="D114" t="inlineStr"/>
+        <v>46</v>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>pier_2_surf</t>
+        </is>
+      </c>
       <c r="E114" t="inlineStr"/>
       <c r="F114" t="inlineStr"/>
     </row>
@@ -2389,11 +2389,11 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>node</t>
         </is>
       </c>
       <c r="C115" t="n">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="D115" t="inlineStr"/>
       <c r="E115" t="inlineStr"/>
@@ -2409,7 +2409,7 @@
         </is>
       </c>
       <c r="C116" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="D116" t="inlineStr"/>
       <c r="E116" t="inlineStr"/>
@@ -2421,11 +2421,11 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>element</t>
+          <t>node</t>
         </is>
       </c>
       <c r="C117" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="D117" t="inlineStr"/>
       <c r="E117" t="inlineStr"/>
@@ -2441,7 +2441,7 @@
         </is>
       </c>
       <c r="C118" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="D118" t="inlineStr"/>
       <c r="E118" t="inlineStr"/>
@@ -2453,11 +2453,11 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>node</t>
+          <t>element</t>
         </is>
       </c>
       <c r="C119" t="n">
-        <v>30</v>
+        <v>2</v>
       </c>
       <c r="D119" t="inlineStr"/>
       <c r="E119" t="inlineStr"/>
@@ -2473,7 +2473,7 @@
         </is>
       </c>
       <c r="C120" t="n">
-        <v>15</v>
+        <v>55</v>
       </c>
       <c r="D120" t="inlineStr"/>
       <c r="E120" t="inlineStr"/>
@@ -2489,7 +2489,7 @@
         </is>
       </c>
       <c r="C121" t="n">
-        <v>27</v>
+        <v>40</v>
       </c>
       <c r="D121" t="inlineStr"/>
       <c r="E121" t="inlineStr"/>
@@ -2505,7 +2505,7 @@
         </is>
       </c>
       <c r="C122" t="n">
-        <v>10</v>
+        <v>35</v>
       </c>
       <c r="D122" t="inlineStr"/>
       <c r="E122" t="inlineStr"/>
@@ -2521,27 +2521,11 @@
         </is>
       </c>
       <c r="C123" t="n">
-        <v>53</v>
+        <v>18</v>
       </c>
       <c r="D123" t="inlineStr"/>
       <c r="E123" t="inlineStr"/>
       <c r="F123" t="inlineStr"/>
-    </row>
-    <row r="124">
-      <c r="A124" t="n">
-        <v>122</v>
-      </c>
-      <c r="B124" t="inlineStr">
-        <is>
-          <t>element</t>
-        </is>
-      </c>
-      <c r="C124" t="n">
-        <v>36</v>
-      </c>
-      <c r="D124" t="inlineStr"/>
-      <c r="E124" t="inlineStr"/>
-      <c r="F124" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>